<commit_message>
Fix exportacion de plantilla de kardex, busqueda por filtros y diseño de tablas
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_productos_general_o_categoria.xlsx
+++ b/public/templates/plantilla_productos_general_o_categoria.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rengifo\Desktop\Proyectos\sistema_de_inventario-rengifo-ltda\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E0222C3-8E33-4A55-9FA6-AACD0C92008E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE829E22-D66A-44E0-BD2A-D62FFE0465AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{29730ABD-B3A1-4C07-BD99-22D4B675851D}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
   <si>
     <t>Nombre de la empresa</t>
   </si>
@@ -105,6 +105,9 @@
   </si>
   <si>
     <t>NOMBRE</t>
+  </si>
+  <si>
+    <t>MARCA</t>
   </si>
 </sst>
 </file>
@@ -186,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -308,11 +311,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -320,6 +349,8 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -338,17 +369,22 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -357,17 +393,20 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -702,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8ACB6CE-280D-4ED1-9FCF-A25BA70014F9}">
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
@@ -725,19 +764,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
@@ -746,21 +785,21 @@
       <c r="Q1" s="1"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="19" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
       <c r="L2" s="2"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
@@ -769,21 +808,21 @@
       <c r="Q2" s="1"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="20" t="s">
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
@@ -792,19 +831,19 @@
       <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="21" t="s">
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
@@ -813,19 +852,19 @@
       <c r="Q4" s="1"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
@@ -834,17 +873,17 @@
       <c r="Q5" s="1"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
@@ -853,19 +892,19 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
@@ -874,17 +913,17 @@
       <c r="Q7" s="1"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
@@ -893,19 +932,19 @@
       <c r="Q8" s="1"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
@@ -933,134 +972,399 @@
       <c r="Q10" s="1"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="5" t="s">
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="4" t="s">
+      <c r="G11" s="8"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4" t="s">
+      <c r="K11" s="18"/>
+      <c r="L11" s="18"/>
+      <c r="M11" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
-      <c r="P11" s="4" t="s">
+      <c r="N11" s="18"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="Q11" s="4"/>
+      <c r="Q11" s="18"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="11" t="s">
+      <c r="A12" s="18"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K12" s="11" t="s">
+      <c r="K12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L12" s="11" t="s">
+      <c r="L12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M12" s="11" t="s">
+      <c r="M12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="N12" s="11" t="s">
+      <c r="N12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="O12" s="11" t="s">
+      <c r="O12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="P12" s="11" t="s">
+      <c r="P12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="Q12" s="11" t="s">
+      <c r="Q12" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
-      <c r="N13" s="12"/>
-      <c r="O13" s="12"/>
-      <c r="P13" s="12"/>
-      <c r="Q13" s="12"/>
+      <c r="A13" s="22"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="22"/>
+      <c r="Q13" s="22"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="12"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="12" t="s">
+      <c r="A14" s="22"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="J14" s="12">
+      <c r="J14" s="22">
         <v>0</v>
       </c>
-      <c r="K14" s="12" t="s">
+      <c r="K14" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="L14" s="12">
+      <c r="L14" s="22">
         <v>0</v>
       </c>
-      <c r="M14" s="12">
+      <c r="M14" s="22">
         <v>0</v>
       </c>
-      <c r="N14" s="12" t="s">
+      <c r="N14" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="O14" s="12">
+      <c r="O14" s="22">
         <v>0</v>
       </c>
-      <c r="P14" s="12">
+      <c r="P14" s="22">
         <v>0</v>
       </c>
-      <c r="Q14" s="12">
+      <c r="Q14" s="22">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" s="21"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="21"/>
+      <c r="I15" s="21"/>
+      <c r="J15" s="21"/>
+      <c r="K15" s="21"/>
+      <c r="L15" s="21"/>
+      <c r="M15" s="21"/>
+      <c r="N15" s="21"/>
+      <c r="O15" s="21"/>
+      <c r="P15" s="21"/>
+      <c r="Q15" s="21"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="21"/>
+      <c r="I16" s="21"/>
+      <c r="J16" s="21"/>
+      <c r="K16" s="21"/>
+      <c r="L16" s="21"/>
+      <c r="M16" s="21"/>
+      <c r="N16" s="21"/>
+      <c r="O16" s="21"/>
+      <c r="P16" s="21"/>
+      <c r="Q16" s="21"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="21"/>
+      <c r="K17" s="21"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="21"/>
+      <c r="N17" s="21"/>
+      <c r="O17" s="21"/>
+      <c r="P17" s="21"/>
+      <c r="Q17" s="21"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" s="21"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="21"/>
+      <c r="P18" s="21"/>
+      <c r="Q18" s="21"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A19" s="21"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="21"/>
+      <c r="K19" s="21"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="21"/>
+      <c r="O19" s="21"/>
+      <c r="P19" s="21"/>
+      <c r="Q19" s="21"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A20" s="21"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="21"/>
+      <c r="L20" s="21"/>
+      <c r="M20" s="21"/>
+      <c r="N20" s="21"/>
+      <c r="O20" s="21"/>
+      <c r="P20" s="21"/>
+      <c r="Q20" s="21"/>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A21" s="21"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="21"/>
+      <c r="H21" s="21"/>
       <c r="I21" s="3"/>
+      <c r="J21" s="21"/>
+      <c r="K21" s="21"/>
+      <c r="L21" s="21"/>
+      <c r="M21" s="21"/>
+      <c r="N21" s="21"/>
+      <c r="O21" s="21"/>
+      <c r="P21" s="21"/>
+      <c r="Q21" s="21"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A22" s="21"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="21"/>
+      <c r="L22" s="21"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
+      <c r="O22" s="21"/>
+      <c r="P22" s="21"/>
+      <c r="Q22" s="21"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A23" s="21"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="21"/>
+      <c r="L23" s="21"/>
+      <c r="M23" s="21"/>
+      <c r="N23" s="21"/>
+      <c r="O23" s="21"/>
+      <c r="P23" s="21"/>
+      <c r="Q23" s="21"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A24" s="21"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="21"/>
+      <c r="K24" s="21"/>
+      <c r="L24" s="21"/>
+      <c r="M24" s="21"/>
+      <c r="N24" s="21"/>
+      <c r="O24" s="21"/>
+      <c r="P24" s="21"/>
+      <c r="Q24" s="21"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A25" s="21"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="21"/>
+      <c r="K25" s="21"/>
+      <c r="L25" s="21"/>
+      <c r="M25" s="21"/>
+      <c r="N25" s="21"/>
+      <c r="O25" s="21"/>
+      <c r="P25" s="21"/>
+      <c r="Q25" s="21"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A26" s="21"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="21"/>
+      <c r="K26" s="21"/>
+      <c r="L26" s="21"/>
+      <c r="M26" s="21"/>
+      <c r="N26" s="21"/>
+      <c r="O26" s="21"/>
+      <c r="P26" s="21"/>
+      <c r="Q26" s="21"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A27" s="21"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="21"/>
+      <c r="L27" s="21"/>
+      <c r="M27" s="21"/>
+      <c r="N27" s="21"/>
+      <c r="O27" s="21"/>
+      <c r="P27" s="21"/>
+      <c r="Q27" s="21"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A28" s="21"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="21"/>
+      <c r="K28" s="21"/>
+      <c r="L28" s="21"/>
+      <c r="M28" s="21"/>
+      <c r="N28" s="21"/>
+      <c r="O28" s="21"/>
+      <c r="P28" s="21"/>
+      <c r="Q28" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="25">
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A11:A12"/>
@@ -1070,23 +1374,24 @@
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A6:C6"/>
+    <mergeCell ref="C7:F7"/>
     <mergeCell ref="G2:K2"/>
     <mergeCell ref="G3:K3"/>
     <mergeCell ref="G4:K4"/>
     <mergeCell ref="M11:O11"/>
     <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="B11:E12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="C7:F7"/>
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="I11:I12"/>
     <mergeCell ref="J11:L11"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="F14:H14"/>
     <mergeCell ref="F11:H12"/>
+    <mergeCell ref="B11:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E11:E12"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.74803149606299213" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="85" orientation="landscape" r:id="rId1"/>
+  <pageSetup fitToWidth="0" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix filtros y exportaciones de kardex y productos con plantillas estandarizadas
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_productos_general_o_categoria.xlsx
+++ b/public/templates/plantilla_productos_general_o_categoria.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rengifo\Desktop\Proyectos\sistema_de_inventario-rengifo-ltda\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE829E22-D66A-44E0-BD2A-D62FFE0465AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D094396C-1A2A-490E-A2AB-B1830559B9F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{29730ABD-B3A1-4C07-BD99-22D4B675851D}"/>
   </bookViews>
@@ -341,7 +341,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -351,37 +351,14 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -393,18 +370,40 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -741,7 +740,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8ACB6CE-280D-4ED1-9FCF-A25BA70014F9}">
-  <dimension ref="A1:Q28"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
@@ -764,11 +766,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -785,21 +787,21 @@
       <c r="Q1" s="1"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
       <c r="L2" s="2"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
@@ -808,21 +810,21 @@
       <c r="Q2" s="1"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
@@ -831,19 +833,19 @@
       <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
-      <c r="G4" s="17" t="s">
+      <c r="G4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
@@ -852,11 +854,11 @@
       <c r="Q4" s="1"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
@@ -873,9 +875,9 @@
       <c r="Q5" s="1"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="20"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -892,14 +894,14 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
       <c r="G7" s="5"/>
       <c r="H7" s="6"/>
       <c r="I7" s="5"/>
@@ -932,15 +934,15 @@
       <c r="Q8" s="1"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
@@ -972,50 +974,50 @@
       <c r="Q10" s="1"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="13" t="s">
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="8"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="18" t="s">
+      <c r="G11" s="19"/>
+      <c r="H11" s="20"/>
+      <c r="I11" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J11" s="18" t="s">
+      <c r="J11" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="K11" s="18"/>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18" t="s">
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="18"/>
-      <c r="O11" s="18"/>
-      <c r="P11" s="18" t="s">
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="Q11" s="18"/>
+      <c r="Q11" s="11"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="18"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="18"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="11"/>
       <c r="J12" s="4" t="s">
         <v>10</v>
       </c>
@@ -1042,329 +1044,81 @@
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="22"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="22"/>
-      <c r="L13" s="22"/>
-      <c r="M13" s="22"/>
-      <c r="N13" s="22"/>
-      <c r="O13" s="22"/>
-      <c r="P13" s="22"/>
-      <c r="Q13" s="22"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
+      <c r="Q13" s="7"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="22"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="22" t="s">
+      <c r="A14" s="7"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J14" s="22">
+      <c r="J14" s="7">
         <v>0</v>
       </c>
-      <c r="K14" s="22" t="s">
+      <c r="K14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L14" s="22">
+      <c r="L14" s="7">
         <v>0</v>
       </c>
-      <c r="M14" s="22">
+      <c r="M14" s="7">
         <v>0</v>
       </c>
-      <c r="N14" s="22" t="s">
+      <c r="N14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="O14" s="22">
+      <c r="O14" s="7">
         <v>0</v>
       </c>
-      <c r="P14" s="22">
+      <c r="P14" s="7">
         <v>0</v>
       </c>
-      <c r="Q14" s="22">
+      <c r="Q14" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A15" s="21"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="21"/>
-      <c r="L15" s="21"/>
-      <c r="M15" s="21"/>
-      <c r="N15" s="21"/>
-      <c r="O15" s="21"/>
-      <c r="P15" s="21"/>
-      <c r="Q15" s="21"/>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="21"/>
-      <c r="O16" s="21"/>
-      <c r="P16" s="21"/>
-      <c r="Q16" s="21"/>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="21"/>
-      <c r="L17" s="21"/>
-      <c r="M17" s="21"/>
-      <c r="N17" s="21"/>
-      <c r="O17" s="21"/>
-      <c r="P17" s="21"/>
-      <c r="Q17" s="21"/>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A18" s="21"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21"/>
-      <c r="M18" s="21"/>
-      <c r="N18" s="21"/>
-      <c r="O18" s="21"/>
-      <c r="P18" s="21"/>
-      <c r="Q18" s="21"/>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A19" s="21"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="21"/>
-      <c r="H19" s="21"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="21"/>
-      <c r="K19" s="21"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="21"/>
-      <c r="N19" s="21"/>
-      <c r="O19" s="21"/>
-      <c r="P19" s="21"/>
-      <c r="Q19" s="21"/>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A20" s="21"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
-      <c r="L20" s="21"/>
-      <c r="M20" s="21"/>
-      <c r="N20" s="21"/>
-      <c r="O20" s="21"/>
-      <c r="P20" s="21"/>
-      <c r="Q20" s="21"/>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A21" s="21"/>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
+    <row r="21" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I21" s="3"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="21"/>
-      <c r="N21" s="21"/>
-      <c r="O21" s="21"/>
-      <c r="P21" s="21"/>
-      <c r="Q21" s="21"/>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A22" s="21"/>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21"/>
-      <c r="M22" s="21"/>
-      <c r="N22" s="21"/>
-      <c r="O22" s="21"/>
-      <c r="P22" s="21"/>
-      <c r="Q22" s="21"/>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A23" s="21"/>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="21"/>
-      <c r="L23" s="21"/>
-      <c r="M23" s="21"/>
-      <c r="N23" s="21"/>
-      <c r="O23" s="21"/>
-      <c r="P23" s="21"/>
-      <c r="Q23" s="21"/>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A24" s="21"/>
-      <c r="B24" s="21"/>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
-      <c r="J24" s="21"/>
-      <c r="K24" s="21"/>
-      <c r="L24" s="21"/>
-      <c r="M24" s="21"/>
-      <c r="N24" s="21"/>
-      <c r="O24" s="21"/>
-      <c r="P24" s="21"/>
-      <c r="Q24" s="21"/>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A25" s="21"/>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="21"/>
-      <c r="K25" s="21"/>
-      <c r="L25" s="21"/>
-      <c r="M25" s="21"/>
-      <c r="N25" s="21"/>
-      <c r="O25" s="21"/>
-      <c r="P25" s="21"/>
-      <c r="Q25" s="21"/>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A26" s="21"/>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
-      <c r="I26" s="21"/>
-      <c r="J26" s="21"/>
-      <c r="K26" s="21"/>
-      <c r="L26" s="21"/>
-      <c r="M26" s="21"/>
-      <c r="N26" s="21"/>
-      <c r="O26" s="21"/>
-      <c r="P26" s="21"/>
-      <c r="Q26" s="21"/>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A27" s="21"/>
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="21"/>
-      <c r="I27" s="21"/>
-      <c r="J27" s="21"/>
-      <c r="K27" s="21"/>
-      <c r="L27" s="21"/>
-      <c r="M27" s="21"/>
-      <c r="N27" s="21"/>
-      <c r="O27" s="21"/>
-      <c r="P27" s="21"/>
-      <c r="Q27" s="21"/>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A28" s="21"/>
-      <c r="B28" s="21"/>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="21"/>
-      <c r="J28" s="21"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="21"/>
-      <c r="M28" s="21"/>
-      <c r="N28" s="21"/>
-      <c r="O28" s="21"/>
-      <c r="P28" s="21"/>
-      <c r="Q28" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="F11:H12"/>
+    <mergeCell ref="B11:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="P11:Q11"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:L11"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A11:A12"/>
@@ -1375,23 +1129,8 @@
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="C7:F7"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F11:H12"/>
-    <mergeCell ref="B11:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E11:E12"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.74803149606299213" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup fitToWidth="0" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>